<commit_message>
Laminas nacionales nuevas (Por region, piramides por region), texto delante de cada lamina y bajas de laminas legacy
</commit_message>
<xml_diff>
--- a/output/graficos_nacionales/plot_nacional_regiones_d_deptot_a_2018.xlsx
+++ b/output/graficos_nacionales/plot_nacional_regiones_d_deptot_a_2018.xlsx
@@ -10,75 +10,78 @@
     <sheet name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Regiones'!$A$1:$B$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Regiones'!$A$1:$B$18</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
-  <si>
-    <t xml:space="preserve">Región</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+  <si>
+    <t xml:space="preserve">Territorio</t>
   </si>
   <si>
     <t xml:space="preserve">Valor</t>
   </si>
   <si>
+    <t xml:space="preserve">Chile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arica y Parinacota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Araucanía</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los Ríos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valparaíso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ñuble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coquimbo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magallanes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O'Higgins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biobío</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aysén</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atacama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los Lagos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarapacá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metropolitana</t>
+  </si>
+  <si>
     <t xml:space="preserve">Antofagasta</t>
   </si>
   <si>
-    <t xml:space="preserve">Arica y Parinacota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atacama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aysén</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biobío</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coquimbo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Araucanía</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los Lagos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los Ríos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Magallanes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metropolitana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O'Higgins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarapacá</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valparaíso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ñuble</t>
-  </si>
-  <si>
     <t xml:space="preserve">Campo</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-16 21:06</t>
+    <t xml:space="preserve">2026-10-01 00:50</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -490,7 +493,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>50.29</v>
+        <v>57.06</v>
       </c>
     </row>
     <row r="3">
@@ -506,7 +509,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>55.71</v>
+        <v>60.21</v>
       </c>
     </row>
     <row r="5">
@@ -514,7 +517,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>56.2</v>
+        <v>59.08</v>
       </c>
     </row>
     <row r="6">
@@ -522,7 +525,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>56.21</v>
+        <v>58.72</v>
       </c>
     </row>
     <row r="7">
@@ -530,7 +533,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>57.67</v>
+        <v>58.55</v>
       </c>
     </row>
     <row r="8">
@@ -538,7 +541,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>60.21</v>
+        <v>57.67</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +549,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>54.68</v>
+        <v>57.17</v>
       </c>
     </row>
     <row r="10">
@@ -554,7 +557,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>59.08</v>
+        <v>57.13</v>
       </c>
     </row>
     <row r="11">
@@ -562,7 +565,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>57.13</v>
+        <v>56.99</v>
       </c>
     </row>
     <row r="12">
@@ -570,7 +573,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>57.17</v>
+        <v>56.21</v>
       </c>
     </row>
     <row r="13">
@@ -578,7 +581,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>52.36</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="14">
@@ -586,7 +589,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>56.99</v>
+        <v>55.71</v>
       </c>
     </row>
     <row r="15">
@@ -594,7 +597,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>54.56</v>
+        <v>54.68</v>
       </c>
     </row>
     <row r="16">
@@ -602,7 +605,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>58.72</v>
+        <v>54.56</v>
       </c>
     </row>
     <row r="17">
@@ -610,11 +613,19 @@
         <v>17</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>58.55</v>
+        <v>52.36</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>50.29</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B17"/>
+  <autoFilter ref="A1:B18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -631,7 +642,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -639,50 +650,50 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>